<commit_message>
refactor: move shared diagram rules to static defaults
Use the built-in shape and line registries as the fallback for every workbook, while allowing workbook rows to override them. Remove duplicated rule sheets from the approved samples, preserve pristine backups, and add an idempotent cleanup utility plus regression coverage.
</commit_message>
<xml_diff>
--- a/webapp/backend/samples/TAKSY_VPM_Landscape_v3.xlsx
+++ b/webapp/backend/samples/TAKSY_VPM_Landscape_v3.xlsx
@@ -9,17 +9,15 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How_To" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shape_Library" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Line_Rules" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diagrams" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nodes" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diagrams" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nodes" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edges" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Shape_Library'!$A$1:$K$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Line_Rules'!$A$1:$J$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Diagrams'!$A$1:$F$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Nodes'!$A$1:$K$33</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Edges'!$A$1:$G$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Diagrams'!$A$1:$F$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Nodes'!$A$1:$K$33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Edges'!$A$1:$G$39</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -548,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -624,194 +622,47 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>group</t>
+          <t>bus_lane</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>EA</t>
+          <t>Network</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>rectangle, dashed</t>
+          <t>rectangle</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
+        <v>1700</v>
+      </c>
+      <c r="E2" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="F2" s="5" t="n">
         <v>400</v>
       </c>
-      <c r="E2" s="5" t="n">
-        <v>300</v>
-      </c>
-      <c r="F2" s="5" t="n">
-        <v>200</v>
-      </c>
       <c r="G2" s="5" t="n">
-        <v>150</v>
+        <v>36</v>
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>#FFFFFF</t>
+          <t>#EAF6FB</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
         <is>
-          <t>#808080</t>
+          <t>#4A90B8</t>
         </is>
       </c>
       <c r="J2" s="5" t="inlineStr">
         <is>
-          <t>container</t>
+          <t>N</t>
         </is>
       </c>
       <c r="K2" s="5" t="inlineStr">
-        <is>
-          <t>Generic container; size from children</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>application_component</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>EA</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>rectangle</t>
-        </is>
-      </c>
-      <c r="D3" s="5" t="n">
-        <v>150</v>
-      </c>
-      <c r="E3" s="5" t="n">
-        <v>55</v>
-      </c>
-      <c r="F3" s="5" t="n">
-        <v>110</v>
-      </c>
-      <c r="G3" s="5" t="n">
-        <v>45</v>
-      </c>
-      <c r="H3" s="5" t="inlineStr">
-        <is>
-          <t>#DAE8FC</t>
-        </is>
-      </c>
-      <c r="I3" s="5" t="inlineStr">
-        <is>
-          <t>#4A7EBB</t>
-        </is>
-      </c>
-      <c r="J3" s="5" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K3" s="5" t="inlineStr">
-        <is>
-          <t>Standard system/module box</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>database</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>EA</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>cylinder</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="n">
-        <v>130</v>
-      </c>
-      <c r="E4" s="5" t="n">
-        <v>70</v>
-      </c>
-      <c r="F4" s="5" t="n">
-        <v>100</v>
-      </c>
-      <c r="G4" s="5" t="n">
-        <v>60</v>
-      </c>
-      <c r="H4" s="5" t="inlineStr">
-        <is>
-          <t>#E1D5E7</t>
-        </is>
-      </c>
-      <c r="I4" s="5" t="inlineStr">
-        <is>
-          <t>#9673A6</t>
-        </is>
-      </c>
-      <c r="J4" s="5" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K4" s="5" t="inlineStr">
-        <is>
-          <t>Data store</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>bus_lane</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>Network</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>rectangle</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="n">
-        <v>1700</v>
-      </c>
-      <c r="E5" s="5" t="n">
-        <v>40</v>
-      </c>
-      <c r="F5" s="5" t="n">
-        <v>400</v>
-      </c>
-      <c r="G5" s="5" t="n">
-        <v>36</v>
-      </c>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>#EAF6FB</t>
-        </is>
-      </c>
-      <c r="I5" s="5" t="inlineStr">
-        <is>
-          <t>#4A90B8</t>
-        </is>
-      </c>
-      <c r="J5" s="5" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K5" s="5" t="inlineStr">
         <is>
           <t>Wide horizontal integration bus (AIN)</t>
         </is>
@@ -824,185 +675,6 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:J3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="9" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="40" customWidth="1" min="10" max="10"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>relation_type</t>
-        </is>
-      </c>
-      <c r="B1" s="4" t="inlineStr">
-        <is>
-          <t>family</t>
-        </is>
-      </c>
-      <c r="C1" s="4" t="inlineStr">
-        <is>
-          <t>line_style</t>
-        </is>
-      </c>
-      <c r="D1" s="4" t="inlineStr">
-        <is>
-          <t>width_px</t>
-        </is>
-      </c>
-      <c r="E1" s="4" t="inlineStr">
-        <is>
-          <t>source_end</t>
-        </is>
-      </c>
-      <c r="F1" s="4" t="inlineStr">
-        <is>
-          <t>target_end</t>
-        </is>
-      </c>
-      <c r="G1" s="4" t="inlineStr">
-        <is>
-          <t>routing</t>
-        </is>
-      </c>
-      <c r="H1" s="4" t="inlineStr">
-        <is>
-          <t>label_position</t>
-        </is>
-      </c>
-      <c r="I1" s="4" t="inlineStr">
-        <is>
-          <t>color_hex</t>
-        </is>
-      </c>
-      <c r="J1" s="4" t="inlineStr">
-        <is>
-          <t>notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="5" t="inlineStr">
-        <is>
-          <t>data_flow</t>
-        </is>
-      </c>
-      <c r="B2" s="5" t="inlineStr">
-        <is>
-          <t>EA</t>
-        </is>
-      </c>
-      <c r="C2" s="5" t="inlineStr">
-        <is>
-          <t>solid</t>
-        </is>
-      </c>
-      <c r="D2" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E2" s="5" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F2" s="5" t="inlineStr">
-        <is>
-          <t>open arrow</t>
-        </is>
-      </c>
-      <c r="G2" s="5" t="inlineStr">
-        <is>
-          <t>orthogonal</t>
-        </is>
-      </c>
-      <c r="H2" s="5" t="inlineStr">
-        <is>
-          <t>midpoint</t>
-        </is>
-      </c>
-      <c r="I2" s="5" t="inlineStr">
-        <is>
-          <t>#3B6EA8</t>
-        </is>
-      </c>
-      <c r="J2" s="5" t="inlineStr">
-        <is>
-          <t>Numbered integration/interface reference</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>association</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>EA</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>solid</t>
-        </is>
-      </c>
-      <c r="D3" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E3" s="5" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F3" s="5" t="inlineStr">
-        <is>
-          <t>open arrow</t>
-        </is>
-      </c>
-      <c r="G3" s="5" t="inlineStr">
-        <is>
-          <t>orthogonal</t>
-        </is>
-      </c>
-      <c r="H3" s="5" t="inlineStr">
-        <is>
-          <t>midpoint</t>
-        </is>
-      </c>
-      <c r="I3" s="5" t="inlineStr">
-        <is>
-          <t>#666666</t>
-        </is>
-      </c>
-      <c r="J3" s="5" t="inlineStr">
-        <is>
-          <t>Generic link</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:J3"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1089,7 +761,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2488,7 +2160,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>